<commit_message>
fix resident excel template
</commit_message>
<xml_diff>
--- a/frontend/public/excel/resident_import_template.xlsx
+++ b/frontend/public/excel/resident_import_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Docs\sdx\room-management-system\frontend\public\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{097032E6-52EB-4218-9985-2EB906B869BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94432F48-55EF-4591-AB32-3480BCDBA68F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{BF556505-7D98-4BFA-ACA6-CE19601E0DE6}"/>
+    <workbookView xWindow="1980" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{BF556505-7D98-4BFA-ACA6-CE19601E0DE6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>fullName</t>
   </si>
@@ -84,6 +84,18 @@
   </si>
   <si>
     <t>phone</t>
+  </si>
+  <si>
+    <t>mealType</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>MALE</t>
+  </si>
+  <si>
+    <t>western</t>
   </si>
 </sst>
 </file>
@@ -466,14 +478,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C57804A-CCBE-4D5B-B2EC-DDB9C151A1D8}">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="13.109375" customWidth="1"/>
     <col min="3" max="3" width="13.5546875" customWidth="1"/>
     <col min="4" max="4" width="14.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -481,53 +494,65 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>14</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E2">
         <v>12345678</v>
       </c>
-      <c r="D2">
+      <c r="F2">
         <v>98628172291</v>
-      </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
       </c>
       <c r="G2" t="s">
         <v>10</v>
       </c>
       <c r="H2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" t="s">
         <v>12</v>
       </c>
-      <c r="I2" t="s">
+      <c r="K2" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>